<commit_message>
BMP site: Survey123 certification as a checkbox, Connect notes
Survey123 has no acknowledge question type, so Connect rendered the
maintenance form's certification as an unsupported trigger with no label.
It is now a required single-choice select_multiple. FORMS.md and the
project note record how Connect copies and locks the XLSForm and that both
surveys were created in Connect on Oct. 21, 2026, unpublished.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/qa/bmp/forms/survey123/bmp-maintenance-documentation.xlsx
+++ b/qa/bmp/forms/survey123/bmp-maintenance-documentation.xlsx
@@ -424,10 +424,10 @@
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="70" customWidth="1" min="3" max="3"/>
+    <col width="51" customWidth="1" min="3" max="3"/>
     <col width="70" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="42" customWidth="1" min="6" max="6"/>
     <col width="70" customWidth="1" min="7" max="7"/>
     <col width="70" customWidth="1" min="8" max="8"/>
     <col width="70" customWidth="1" min="9" max="9"/>
@@ -1599,7 +1599,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>acknowledge</t>
+          <t>select_multiple certify</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1609,7 +1609,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>I certify that the information in this form is accurate and that I am authorized to submit it for this property.</t>
+          <t>Certification</t>
         </is>
       </c>
       <c r="D33" t="inlineStr"/>
@@ -1618,7 +1618,11 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="F33" t="inlineStr"/>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>Check the box to certify the submission.</t>
+        </is>
+      </c>
       <c r="G33" t="inlineStr"/>
       <c r="H33" t="inlineStr"/>
       <c r="I33" t="inlineStr"/>
@@ -1641,12 +1645,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C29"/>
+  <dimension ref="A1:C30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
-    <col width="65" customWidth="1" min="3" max="3"/>
+    <col width="70" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2139,6 +2143,23 @@
       <c r="C29" t="inlineStr">
         <is>
           <t>Other (describe below)</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>certify</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>I certify that the information in this form is accurate and that I am authorized to submit it for this property.</t>
         </is>
       </c>
     </row>

</xml_diff>